<commit_message>
Update the recalibrated transient WVP coefficients
Calibrated with the series head loss (series_dp_ref_m, series_flow_ref_m3_per_h,
series_growth_per_m3) per strang. The initial R_bed_12C_d_per_m row in
strang_props7.csv is derived from these coefficients (initial_bed_resistances).
</commit_message>
<xml_diff>
--- a/productiecapaciteit/results/Wvptweerstand/Wvptweerstand_modelcoefficienten.xlsx
+++ b/productiecapaciteit/results/Wvptweerstand/Wvptweerstand_modelcoefficienten.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>137.9848283206014</v>
+        <v>155.0853530665898</v>
       </c>
     </row>
     <row r="3">
@@ -569,17 +569,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>405.3146362796253</v>
+        <v>236.5061813767973</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>369.2854774999998</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.399619914777114e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38020965278</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65970960559</v>
       </c>
     </row>
   </sheetData>
@@ -593,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,7 +648,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>99.77931505959782</v>
+        <v>114.4234769440508</v>
       </c>
     </row>
     <row r="3">
@@ -710,17 +750,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>85.5618809546921</v>
+        <v>69.16463646676293</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>312.5833333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4.150427388353646e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38285495371</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66032459941</v>
       </c>
     </row>
   </sheetData>
@@ -734,7 +814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -749,7 +829,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86.79962464158727</v>
+        <v>103.3521203820786</v>
       </c>
     </row>
     <row r="3">
@@ -851,17 +931,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>104.6984005043563</v>
+        <v>53.39498620144901</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>260.1683545833333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.133412705471005e-07</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38315274305</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66036840625</v>
       </c>
     </row>
   </sheetData>
@@ -875,7 +995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -890,7 +1010,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112.7136066826703</v>
+        <v>152.4250464563878</v>
       </c>
     </row>
     <row r="3">
@@ -992,17 +1112,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>99999.99999999984</v>
+        <v>99999.99999976643</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>367.25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.505731836976018e-07</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38365194444</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66042630199</v>
       </c>
     </row>
   </sheetData>
@@ -1016,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,7 +1191,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54.49438930065518</v>
+        <v>85.17427109528553</v>
       </c>
     </row>
     <row r="3">
@@ -1133,17 +1293,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>292.5230342453905</v>
+        <v>99999.99988701307</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>195.9166666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.108117633324632e-07</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38377106481</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.6604864552</v>
       </c>
     </row>
   </sheetData>
@@ -1157,7 +1357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1172,7 +1372,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74.9030607049535</v>
+        <v>97.8644646547428</v>
       </c>
     </row>
     <row r="3">
@@ -1274,17 +1474,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>31.96280993848053</v>
+        <v>27.91689479763951</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>253.6666666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5.99451368478002e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38386960648</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66052055982</v>
       </c>
     </row>
   </sheetData>
@@ -1298,7 +1538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1313,7 +1553,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68.83639703113577</v>
+        <v>81.7734578046211</v>
       </c>
     </row>
     <row r="3">
@@ -1415,17 +1655,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>29.44348931263039</v>
+        <v>23.12781551623712</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>252.7583333333334</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.845970541787556e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38397108796</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66056408199</v>
       </c>
     </row>
   </sheetData>
@@ -1439,7 +1719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1454,7 +1734,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71.22201669341598</v>
+        <v>86.89800830935012</v>
       </c>
     </row>
     <row r="3">
@@ -1556,17 +1836,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48.12182209451906</v>
+        <v>44.10955422856618</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>244.25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6.865851485947927e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38408188657</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66060678982</v>
       </c>
     </row>
   </sheetData>
@@ -1580,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1595,7 +1915,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>52.26551966738259</v>
+        <v>63.19390145362059</v>
       </c>
     </row>
     <row r="3">
@@ -1697,17 +2017,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>60.45198865816435</v>
+        <v>54.9438936012447</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>256.3333333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>9.831147229113991e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38421917824</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66064773737</v>
       </c>
     </row>
   </sheetData>
@@ -1721,7 +2081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1736,7 +2096,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43.59566385278046</v>
+        <v>47.69317896012079</v>
       </c>
     </row>
     <row r="3">
@@ -1838,17 +2198,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>219.3429509924534</v>
+        <v>4.880712947043902</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>82.26086766666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.492304592100548e-07</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46202.43523520969</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65717731482</v>
       </c>
     </row>
   </sheetData>
@@ -1862,7 +2262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1877,7 +2277,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>93.99272641297553</v>
+        <v>108.5422268907658</v>
       </c>
     </row>
     <row r="3">
@@ -1979,17 +2379,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1136.510113788484</v>
+        <v>2907.028313687438</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>203.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6.157943841314275e-22</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38442649305</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65727664352</v>
       </c>
     </row>
   </sheetData>
@@ -2003,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2018,7 +2458,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>98.74937523490478</v>
+        <v>104.9122344010072</v>
       </c>
     </row>
     <row r="3">
@@ -2120,17 +2560,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>203.2215208231023</v>
+        <v>144.3433084949338</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>448.5833333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4.770706358529135e-09</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38067107639</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65980620577</v>
       </c>
     </row>
   </sheetData>
@@ -2144,7 +2624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2159,7 +2639,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79.36630652693906</v>
+        <v>91.74414939678178</v>
       </c>
     </row>
     <row r="3">
@@ -2261,17 +2741,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>34.25272137327244</v>
+        <v>27.92923130564965</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>273.3333333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7.53728303849933e-17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38451594907</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65732862268</v>
       </c>
     </row>
   </sheetData>
@@ -2285,7 +2805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2300,7 +2820,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74.53299555740928</v>
+        <v>91.93284427380112</v>
       </c>
     </row>
     <row r="3">
@@ -2402,17 +2922,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>29.63604694723997</v>
+        <v>24.47914674987855</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>214.3333333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.400429173613405e-09</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38463738426</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65737655092</v>
       </c>
     </row>
   </sheetData>
@@ -2426,7 +2986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2441,7 +3001,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>78.22770129569565</v>
+        <v>94.33705678283141</v>
       </c>
     </row>
     <row r="3">
@@ -2543,17 +3103,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26.63519176423128</v>
+        <v>21.42401034360849</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.258100318047656e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38471892361</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65741355324</v>
       </c>
     </row>
   </sheetData>
@@ -2567,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2582,7 +3182,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72.68376620087484</v>
+        <v>86.20152736133117</v>
       </c>
     </row>
     <row r="3">
@@ -2684,17 +3284,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22.99097848191633</v>
+        <v>20.0670923651158</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>255.3333333333333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.358449971927711e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38481663194</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65746504629</v>
       </c>
     </row>
   </sheetData>
@@ -2708,7 +3348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2723,7 +3363,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53.97574764488891</v>
+        <v>70.53306015253686</v>
       </c>
     </row>
     <row r="3">
@@ -2825,17 +3465,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>151.5252036597074</v>
+        <v>278.6337552169063</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4.819195104394007e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38487244213</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.6575434375</v>
       </c>
     </row>
   </sheetData>
@@ -2849,7 +3529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2864,7 +3544,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>110.1655139478601</v>
+        <v>121.9392492155175</v>
       </c>
     </row>
     <row r="3">
@@ -2966,17 +3646,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>67.05711947233651</v>
+        <v>56.76703997536914</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6.487673078983902e-09</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38095324074</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65985395746</v>
       </c>
     </row>
   </sheetData>
@@ -2990,7 +3710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3005,7 +3725,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90.29290632316274</v>
+        <v>100.5702100726431</v>
       </c>
     </row>
     <row r="3">
@@ -3107,17 +3827,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>51.38878640149944</v>
+        <v>43.35802790973971</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>348.75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.279646247477633e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38138425926</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65990115407</v>
       </c>
     </row>
   </sheetData>
@@ -3131,7 +3891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3146,7 +3906,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84.07065805081774</v>
+        <v>96.97416085685767</v>
       </c>
     </row>
     <row r="3">
@@ -3248,17 +4008,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>93.66773180416638</v>
+        <v>94.32965824207719</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>395.4166666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.734226403028606e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38159059028</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.65996618004</v>
       </c>
     </row>
   </sheetData>
@@ -3272,7 +4072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3287,7 +4087,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>115.6575917081301</v>
+        <v>137.0423305385885</v>
       </c>
     </row>
     <row r="3">
@@ -3389,17 +4189,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>99999.99999999841</v>
+        <v>99999.99896002925</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>319.1666666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.191806632352289e-07</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38189980324</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66002502797</v>
       </c>
     </row>
   </sheetData>
@@ -3413,7 +4253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3428,7 +4268,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>178.3420989800929</v>
+        <v>209.5964384901635</v>
       </c>
     </row>
     <row r="3">
@@ -3530,17 +4370,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5217.656808069559</v>
+        <v>99999.99389166503</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.454189916668398e-22</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38222395833</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66016261906</v>
       </c>
     </row>
   </sheetData>
@@ -3554,7 +4434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3569,7 +4449,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>117.0730037688785</v>
+        <v>133.4615688277638</v>
       </c>
     </row>
     <row r="3">
@@ -3671,17 +4551,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>179.1142170918835</v>
+        <v>150.2279684346754</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>361.8613256250001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.742955560493003e-08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38242336806</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66022137154</v>
       </c>
     </row>
   </sheetData>
@@ -3695,7 +4615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3710,7 +4630,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>102.0124252150672</v>
+        <v>113.5815174751777</v>
       </c>
     </row>
     <row r="3">
@@ -3812,17 +4732,57 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>65.83201655009906</v>
+        <v>54.93479131902512</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
+          <t>series_dp_ref_m</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>series_flow_ref_m3_per_h</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>391.4166666666667</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>series_datum</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>42005</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>series_growth_per_m3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8.396408716180435e-13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>gewijzigd</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>46200.38261159722</v>
+      <c r="B17" s="2" t="n">
+        <v>46204.66027374272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>